<commit_message>
feat: overheat , Enemy Counter
</commit_message>
<xml_diff>
--- a/Assets/_GraduationProject/02_Feature/02_Character/01_Player/Excel/PlayerSourceMapDatabase.xlsx
+++ b/Assets/_GraduationProject/02_Feature/02_Character/01_Player/Excel/PlayerSourceMapDatabase.xlsx
@@ -106,7 +106,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="0" formatCode=""/>
   </x:numFmts>
-  <x:fonts count="8" x14ac:knownFonts="1">
+  <x:fonts count="9" x14ac:knownFonts="1">
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FF000000"/>
@@ -125,6 +125,13 @@
       <x:name val="돋움"/>
       <x:family val="3"/>
       <x:charset val="129"/>
+    </x:font>
+    <x:font>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
     </x:font>
     <x:font>
       <x:vertAlign val="baseline"/>
@@ -185,9 +192,12 @@
       <x:diagonal/>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="7">
+  <x:cellStyleXfs count="8">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
@@ -546,15 +556,15 @@
   <x:dimension ref="A1:I32"/>
   <x:sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <x:cols>
-    <x:col min="1" max="1" width="21.720625000000002" style="2" customWidth="1"/>
-    <x:col min="2" max="2" width="48.880625" style="2" customWidth="1"/>
-    <x:col min="3" max="3" width="35.360625" style="2" customWidth="1"/>
-    <x:col min="4" max="4" width="13.560625" style="2" customWidth="1"/>
-    <x:col min="5" max="5" width="35.280625" style="2" customWidth="1"/>
-    <x:col min="6" max="6" width="18.010625" style="2" customWidth="1"/>
-    <x:col min="7" max="7" width="18.050625" style="2" customWidth="1"/>
-    <x:col min="8" max="8" width="26.660625" style="2" customWidth="1"/>
-    <x:col min="9" max="9" width="21.310625" style="2" customWidth="1"/>
+    <x:col min="1" max="1" width="17.740625" style="2" customWidth="1"/>
+    <x:col min="2" max="2" width="39.470625" style="2" customWidth="1"/>
+    <x:col min="3" max="3" width="28.650625" style="2" customWidth="1"/>
+    <x:col min="4" max="4" width="11.220625" style="2" customWidth="1"/>
+    <x:col min="5" max="5" width="28.590625" style="2" customWidth="1"/>
+    <x:col min="6" max="6" width="14.770625" style="2" customWidth="1"/>
+    <x:col min="7" max="7" width="14.810625" style="2" customWidth="1"/>
+    <x:col min="8" max="8" width="21.700625" style="2" customWidth="1"/>
+    <x:col min="9" max="9" width="17.410625" style="2" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -603,7 +613,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="F2" s="2" t="n">
-        <x:v>4</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G2" s="2" t="n">
         <x:v>0</x:v>

</xml_diff>